<commit_message>
📊 Full pipeline output Wed May  6 08:13:03 UTC 2026
</commit_message>
<xml_diff>
--- a/output/intraday/dati_intraday_D2_1m_yfinance_2026-05-06.xlsx
+++ b/output/intraday/dati_intraday_D2_1m_yfinance_2026-05-06.xlsx
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G276" t="n">
-        <v>5.34</v>
+        <v>5.35</v>
       </c>
       <c r="H276" t="n">
         <v>5.36</v>
@@ -12572,7 +12572,7 @@
         <v>5.35</v>
       </c>
       <c r="K276" t="n">
-        <v>4687</v>
+        <v>4747</v>
       </c>
       <c r="L276" t="n">
         <v>7.4823</v>
@@ -12868,7 +12868,7 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>5.79</v>
+        <v>5.83</v>
       </c>
       <c r="H283" t="n">
         <v>5.83</v>
@@ -13100,7 +13100,7 @@
         <v>5.71</v>
       </c>
       <c r="K288" t="n">
-        <v>1020</v>
+        <v>1000</v>
       </c>
       <c r="L288" t="n">
         <v>7.4823</v>
@@ -13144,7 +13144,7 @@
         <v>5.68</v>
       </c>
       <c r="K289" t="n">
-        <v>6483</v>
+        <v>6503</v>
       </c>
       <c r="L289" t="n">
         <v>7.4823</v>
@@ -14232,7 +14232,7 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>6.21</v>
+        <v>6.25</v>
       </c>
       <c r="H314" t="n">
         <v>6.25</v>
@@ -15256,7 +15256,7 @@
         <v>6.42</v>
       </c>
       <c r="K337" t="n">
-        <v>10469</v>
+        <v>10470</v>
       </c>
       <c r="L337" t="n">
         <v>7.4823</v>
@@ -15432,7 +15432,7 @@
         <v>6.76</v>
       </c>
       <c r="K341" t="n">
-        <v>2249</v>
+        <v>2160</v>
       </c>
       <c r="L341" t="n">
         <v>7.4823</v>
@@ -15476,7 +15476,7 @@
         <v>6.83</v>
       </c>
       <c r="K342" t="n">
-        <v>4604</v>
+        <v>4693</v>
       </c>
       <c r="L342" t="n">
         <v>7.4823</v>
@@ -20568,7 +20568,7 @@
         </is>
       </c>
       <c r="G458" t="n">
-        <v>6.47</v>
+        <v>6.48</v>
       </c>
       <c r="H458" t="n">
         <v>6.5</v>
@@ -22548,7 +22548,7 @@
         </is>
       </c>
       <c r="G503" t="n">
-        <v>6.88</v>
+        <v>6.93</v>
       </c>
       <c r="H503" t="n">
         <v>6.93</v>
@@ -22856,7 +22856,7 @@
         </is>
       </c>
       <c r="G510" t="n">
-        <v>7.18</v>
+        <v>7.24</v>
       </c>
       <c r="H510" t="n">
         <v>7.24</v>
@@ -23132,7 +23132,7 @@
         <v>7.16</v>
       </c>
       <c r="K516" t="n">
-        <v>11622</v>
+        <v>11531</v>
       </c>
       <c r="L516" t="n">
         <v>7.4823</v>
@@ -23176,7 +23176,7 @@
         <v>7.28</v>
       </c>
       <c r="K517" t="n">
-        <v>5085</v>
+        <v>5176</v>
       </c>
       <c r="L517" t="n">
         <v>7.4823</v>
@@ -24188,7 +24188,7 @@
         <v>7</v>
       </c>
       <c r="K540" t="n">
-        <v>4028</v>
+        <v>3930</v>
       </c>
       <c r="L540" t="n">
         <v>7.4823</v>
@@ -24232,7 +24232,7 @@
         <v>6.94</v>
       </c>
       <c r="K541" t="n">
-        <v>861</v>
+        <v>959</v>
       </c>
       <c r="L541" t="n">
         <v>7.4823</v>
@@ -40116,7 +40116,7 @@
         <v>1.1</v>
       </c>
       <c r="K902" t="n">
-        <v>7558</v>
+        <v>1633166</v>
       </c>
       <c r="L902" t="n">
         <v>1.26</v>
@@ -45120,7 +45120,7 @@
         </is>
       </c>
       <c r="G1016" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="H1016" t="n">
         <v>1.15</v>
@@ -64536,7 +64536,7 @@
         <v>4.87</v>
       </c>
       <c r="K1457" t="n">
-        <v>3444</v>
+        <v>3424</v>
       </c>
       <c r="L1457" t="n">
         <v>4.91</v>
@@ -64580,7 +64580,7 @@
         <v>4.86</v>
       </c>
       <c r="K1458" t="n">
-        <v>4680</v>
+        <v>4700</v>
       </c>
       <c r="L1458" t="n">
         <v>4.91</v>
@@ -65504,7 +65504,7 @@
         <v>9.26</v>
       </c>
       <c r="K1479" t="n">
-        <v>248431</v>
+        <v>248403</v>
       </c>
       <c r="L1479" t="n">
         <v>4.91</v>
@@ -65548,7 +65548,7 @@
         <v>9.550000000000001</v>
       </c>
       <c r="K1480" t="n">
-        <v>285390</v>
+        <v>285418</v>
       </c>
       <c r="L1480" t="n">
         <v>4.91</v>
@@ -65592,7 +65592,7 @@
         <v>9.630000000000001</v>
       </c>
       <c r="K1481" t="n">
-        <v>224699</v>
+        <v>225197</v>
       </c>
       <c r="L1481" t="n">
         <v>4.91</v>
@@ -66032,7 +66032,7 @@
         <v>9.4</v>
       </c>
       <c r="K1491" t="n">
-        <v>211725</v>
+        <v>211714</v>
       </c>
       <c r="L1491" t="n">
         <v>4.91</v>
@@ -66076,7 +66076,7 @@
         <v>9.41</v>
       </c>
       <c r="K1492" t="n">
-        <v>208180</v>
+        <v>208191</v>
       </c>
       <c r="L1492" t="n">
         <v>4.91</v>
@@ -66120,7 +66120,7 @@
         <v>9.07</v>
       </c>
       <c r="K1493" t="n">
-        <v>145808</v>
+        <v>145791</v>
       </c>
       <c r="L1493" t="n">
         <v>4.91</v>
@@ -66164,7 +66164,7 @@
         <v>9.27</v>
       </c>
       <c r="K1494" t="n">
-        <v>60483</v>
+        <v>60500</v>
       </c>
       <c r="L1494" t="n">
         <v>4.91</v>
@@ -66428,7 +66428,7 @@
         <v>9</v>
       </c>
       <c r="K1500" t="n">
-        <v>27266</v>
+        <v>27241</v>
       </c>
       <c r="L1500" t="n">
         <v>4.91</v>
@@ -66472,7 +66472,7 @@
         <v>9.01</v>
       </c>
       <c r="K1501" t="n">
-        <v>67433</v>
+        <v>67458</v>
       </c>
       <c r="L1501" t="n">
         <v>4.91</v>
@@ -67132,7 +67132,7 @@
         <v>10.99</v>
       </c>
       <c r="K1516" t="n">
-        <v>79080</v>
+        <v>79069</v>
       </c>
       <c r="L1516" t="n">
         <v>4.91</v>
@@ -67176,7 +67176,7 @@
         <v>10.8</v>
       </c>
       <c r="K1517" t="n">
-        <v>66291</v>
+        <v>66302</v>
       </c>
       <c r="L1517" t="n">
         <v>4.91</v>
@@ -67560,7 +67560,7 @@
         </is>
       </c>
       <c r="G1526" t="n">
-        <v>9.050000000000001</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="H1526" t="n">
         <v>9.449999999999999</v>
@@ -67616,7 +67616,7 @@
         <v>8.960000000000001</v>
       </c>
       <c r="K1527" t="n">
-        <v>98986</v>
+        <v>98996</v>
       </c>
       <c r="L1527" t="n">
         <v>4.91</v>
@@ -67660,7 +67660,7 @@
         <v>8.27</v>
       </c>
       <c r="K1528" t="n">
-        <v>218590</v>
+        <v>218587</v>
       </c>
       <c r="L1528" t="n">
         <v>4.91</v>
@@ -67704,7 +67704,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="K1529" t="n">
-        <v>307559</v>
+        <v>307562</v>
       </c>
       <c r="L1529" t="n">
         <v>4.91</v>
@@ -67924,7 +67924,7 @@
         <v>8.32</v>
       </c>
       <c r="K1534" t="n">
-        <v>209988</v>
+        <v>210003</v>
       </c>
       <c r="L1534" t="n">
         <v>4.91</v>
@@ -67968,7 +67968,7 @@
         <v>8.31</v>
       </c>
       <c r="K1535" t="n">
-        <v>41090</v>
+        <v>11721801</v>
       </c>
       <c r="L1535" t="n">
         <v>4.91</v>
@@ -68220,7 +68220,7 @@
         </is>
       </c>
       <c r="G1541" t="n">
-        <v>8.51</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="H1541" t="n">
         <v>8.619999999999999</v>
@@ -68232,7 +68232,7 @@
         <v>8.609999999999999</v>
       </c>
       <c r="K1541" t="n">
-        <v>33728</v>
+        <v>34777</v>
       </c>
       <c r="L1541" t="n">
         <v>4.91</v>
@@ -69012,7 +69012,7 @@
         </is>
       </c>
       <c r="G1559" t="n">
-        <v>7.95</v>
+        <v>7.94</v>
       </c>
       <c r="H1559" t="n">
         <v>8.08</v>
@@ -69596,7 +69596,7 @@
         <v>8.1</v>
       </c>
       <c r="K1572" t="n">
-        <v>10574</v>
+        <v>13113558</v>
       </c>
       <c r="L1572" t="n">
         <v>4.91</v>
@@ -74248,13 +74248,13 @@
         </is>
       </c>
       <c r="G1678" t="n">
-        <v>6.93</v>
+        <v>6.85</v>
       </c>
       <c r="H1678" t="n">
-        <v>6.93</v>
+        <v>6.85</v>
       </c>
       <c r="I1678" t="n">
-        <v>6.74</v>
+        <v>6.85</v>
       </c>
       <c r="J1678" t="n">
         <v>6.85</v>
@@ -84028,7 +84028,7 @@
         <v>14.17</v>
       </c>
       <c r="K1900" t="n">
-        <v>5154</v>
+        <v>5104</v>
       </c>
       <c r="L1900" t="n">
         <v>14.5</v>
@@ -84072,7 +84072,7 @@
         <v>14.45</v>
       </c>
       <c r="K1901" t="n">
-        <v>3849</v>
+        <v>3899</v>
       </c>
       <c r="L1901" t="n">
         <v>14.5</v>
@@ -86096,7 +86096,7 @@
         <v>14.04</v>
       </c>
       <c r="K1947" t="n">
-        <v>215</v>
+        <v>167</v>
       </c>
       <c r="L1947" t="n">
         <v>14.5</v>
@@ -86140,7 +86140,7 @@
         <v>14</v>
       </c>
       <c r="K1948" t="n">
-        <v>643</v>
+        <v>691</v>
       </c>
       <c r="L1948" t="n">
         <v>14.5</v>
@@ -87504,7 +87504,7 @@
         <v>14.06</v>
       </c>
       <c r="K1979" t="n">
-        <v>819</v>
+        <v>1289</v>
       </c>
       <c r="L1979" t="n">
         <v>14.5</v>
@@ -88296,7 +88296,7 @@
         <v>14.04</v>
       </c>
       <c r="K1997" t="n">
-        <v>1457</v>
+        <v>1763</v>
       </c>
       <c r="L1997" t="n">
         <v>14.5</v>
@@ -91112,7 +91112,7 @@
         <v>14.11</v>
       </c>
       <c r="K2061" t="n">
-        <v>969</v>
+        <v>953</v>
       </c>
       <c r="L2061" t="n">
         <v>14.5</v>
@@ -91156,7 +91156,7 @@
         <v>14.05</v>
       </c>
       <c r="K2062" t="n">
-        <v>613</v>
+        <v>629</v>
       </c>
       <c r="L2062" t="n">
         <v>14.5</v>
@@ -91860,7 +91860,7 @@
         <v>13.98</v>
       </c>
       <c r="K2078" t="n">
-        <v>7985</v>
+        <v>7907</v>
       </c>
       <c r="L2078" t="n">
         <v>14.5</v>
@@ -91904,7 +91904,7 @@
         <v>13.91</v>
       </c>
       <c r="K2079" t="n">
-        <v>6039</v>
+        <v>6117</v>
       </c>
       <c r="L2079" t="n">
         <v>14.5</v>
@@ -92168,7 +92168,7 @@
         <v>14.17</v>
       </c>
       <c r="K2085" t="n">
-        <v>1364</v>
+        <v>1266</v>
       </c>
       <c r="L2085" t="n">
         <v>14.5</v>
@@ -92212,7 +92212,7 @@
         <v>14.23</v>
       </c>
       <c r="K2086" t="n">
-        <v>14446</v>
+        <v>14544</v>
       </c>
       <c r="L2086" t="n">
         <v>14.5</v>

</xml_diff>

<commit_message>
📊 Full pipeline output Wed May  6 08:36:17 UTC 2026
</commit_message>
<xml_diff>
--- a/output/intraday/dati_intraday_D2_1m_yfinance_2026-05-06.xlsx
+++ b/output/intraday/dati_intraday_D2_1m_yfinance_2026-05-06.xlsx
@@ -12560,7 +12560,7 @@
         </is>
       </c>
       <c r="G276" t="n">
-        <v>5.35</v>
+        <v>5.34</v>
       </c>
       <c r="H276" t="n">
         <v>5.36</v>
@@ -12572,7 +12572,7 @@
         <v>5.35</v>
       </c>
       <c r="K276" t="n">
-        <v>4747</v>
+        <v>4687</v>
       </c>
       <c r="L276" t="n">
         <v>7.4823</v>
@@ -12868,7 +12868,7 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>5.83</v>
+        <v>5.79</v>
       </c>
       <c r="H283" t="n">
         <v>5.83</v>
@@ -13100,7 +13100,7 @@
         <v>5.71</v>
       </c>
       <c r="K288" t="n">
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="L288" t="n">
         <v>7.4823</v>
@@ -13144,7 +13144,7 @@
         <v>5.68</v>
       </c>
       <c r="K289" t="n">
-        <v>6503</v>
+        <v>6483</v>
       </c>
       <c r="L289" t="n">
         <v>7.4823</v>
@@ -14232,7 +14232,7 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>6.25</v>
+        <v>6.21</v>
       </c>
       <c r="H314" t="n">
         <v>6.25</v>
@@ -15256,7 +15256,7 @@
         <v>6.42</v>
       </c>
       <c r="K337" t="n">
-        <v>10470</v>
+        <v>10469</v>
       </c>
       <c r="L337" t="n">
         <v>7.4823</v>
@@ -15432,7 +15432,7 @@
         <v>6.76</v>
       </c>
       <c r="K341" t="n">
-        <v>2160</v>
+        <v>2249</v>
       </c>
       <c r="L341" t="n">
         <v>7.4823</v>
@@ -15476,7 +15476,7 @@
         <v>6.83</v>
       </c>
       <c r="K342" t="n">
-        <v>4693</v>
+        <v>4604</v>
       </c>
       <c r="L342" t="n">
         <v>7.4823</v>
@@ -20568,7 +20568,7 @@
         </is>
       </c>
       <c r="G458" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="H458" t="n">
         <v>6.5</v>
@@ -22548,7 +22548,7 @@
         </is>
       </c>
       <c r="G503" t="n">
-        <v>6.93</v>
+        <v>6.88</v>
       </c>
       <c r="H503" t="n">
         <v>6.93</v>
@@ -22856,7 +22856,7 @@
         </is>
       </c>
       <c r="G510" t="n">
-        <v>7.24</v>
+        <v>7.18</v>
       </c>
       <c r="H510" t="n">
         <v>7.24</v>
@@ -23132,7 +23132,7 @@
         <v>7.16</v>
       </c>
       <c r="K516" t="n">
-        <v>11531</v>
+        <v>11622</v>
       </c>
       <c r="L516" t="n">
         <v>7.4823</v>
@@ -23176,7 +23176,7 @@
         <v>7.28</v>
       </c>
       <c r="K517" t="n">
-        <v>5176</v>
+        <v>5085</v>
       </c>
       <c r="L517" t="n">
         <v>7.4823</v>
@@ -24188,7 +24188,7 @@
         <v>7</v>
       </c>
       <c r="K540" t="n">
-        <v>3930</v>
+        <v>4028</v>
       </c>
       <c r="L540" t="n">
         <v>7.4823</v>
@@ -24232,7 +24232,7 @@
         <v>6.94</v>
       </c>
       <c r="K541" t="n">
-        <v>959</v>
+        <v>861</v>
       </c>
       <c r="L541" t="n">
         <v>7.4823</v>
@@ -40116,7 +40116,7 @@
         <v>1.1</v>
       </c>
       <c r="K902" t="n">
-        <v>1633166</v>
+        <v>7558</v>
       </c>
       <c r="L902" t="n">
         <v>1.26</v>
@@ -45120,7 +45120,7 @@
         </is>
       </c>
       <c r="G1016" t="n">
-        <v>1.14</v>
+        <v>1.15</v>
       </c>
       <c r="H1016" t="n">
         <v>1.15</v>
@@ -64536,7 +64536,7 @@
         <v>4.87</v>
       </c>
       <c r="K1457" t="n">
-        <v>3424</v>
+        <v>3444</v>
       </c>
       <c r="L1457" t="n">
         <v>4.91</v>
@@ -64580,7 +64580,7 @@
         <v>4.86</v>
       </c>
       <c r="K1458" t="n">
-        <v>4700</v>
+        <v>4680</v>
       </c>
       <c r="L1458" t="n">
         <v>4.91</v>
@@ -65504,7 +65504,7 @@
         <v>9.26</v>
       </c>
       <c r="K1479" t="n">
-        <v>248403</v>
+        <v>248431</v>
       </c>
       <c r="L1479" t="n">
         <v>4.91</v>
@@ -65548,7 +65548,7 @@
         <v>9.550000000000001</v>
       </c>
       <c r="K1480" t="n">
-        <v>285418</v>
+        <v>285390</v>
       </c>
       <c r="L1480" t="n">
         <v>4.91</v>
@@ -65592,7 +65592,7 @@
         <v>9.630000000000001</v>
       </c>
       <c r="K1481" t="n">
-        <v>225197</v>
+        <v>224699</v>
       </c>
       <c r="L1481" t="n">
         <v>4.91</v>
@@ -66032,7 +66032,7 @@
         <v>9.4</v>
       </c>
       <c r="K1491" t="n">
-        <v>211714</v>
+        <v>211725</v>
       </c>
       <c r="L1491" t="n">
         <v>4.91</v>
@@ -66076,7 +66076,7 @@
         <v>9.41</v>
       </c>
       <c r="K1492" t="n">
-        <v>208191</v>
+        <v>208180</v>
       </c>
       <c r="L1492" t="n">
         <v>4.91</v>
@@ -66120,7 +66120,7 @@
         <v>9.07</v>
       </c>
       <c r="K1493" t="n">
-        <v>145791</v>
+        <v>145808</v>
       </c>
       <c r="L1493" t="n">
         <v>4.91</v>
@@ -66164,7 +66164,7 @@
         <v>9.27</v>
       </c>
       <c r="K1494" t="n">
-        <v>60500</v>
+        <v>60483</v>
       </c>
       <c r="L1494" t="n">
         <v>4.91</v>
@@ -66428,7 +66428,7 @@
         <v>9</v>
       </c>
       <c r="K1500" t="n">
-        <v>27241</v>
+        <v>27266</v>
       </c>
       <c r="L1500" t="n">
         <v>4.91</v>
@@ -66472,7 +66472,7 @@
         <v>9.01</v>
       </c>
       <c r="K1501" t="n">
-        <v>67458</v>
+        <v>67433</v>
       </c>
       <c r="L1501" t="n">
         <v>4.91</v>
@@ -67132,7 +67132,7 @@
         <v>10.99</v>
       </c>
       <c r="K1516" t="n">
-        <v>79069</v>
+        <v>79080</v>
       </c>
       <c r="L1516" t="n">
         <v>4.91</v>
@@ -67176,7 +67176,7 @@
         <v>10.8</v>
       </c>
       <c r="K1517" t="n">
-        <v>66302</v>
+        <v>66291</v>
       </c>
       <c r="L1517" t="n">
         <v>4.91</v>
@@ -67560,7 +67560,7 @@
         </is>
       </c>
       <c r="G1526" t="n">
-        <v>9.109999999999999</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="H1526" t="n">
         <v>9.449999999999999</v>
@@ -67616,7 +67616,7 @@
         <v>8.960000000000001</v>
       </c>
       <c r="K1527" t="n">
-        <v>98996</v>
+        <v>98986</v>
       </c>
       <c r="L1527" t="n">
         <v>4.91</v>
@@ -67660,7 +67660,7 @@
         <v>8.27</v>
       </c>
       <c r="K1528" t="n">
-        <v>218587</v>
+        <v>218590</v>
       </c>
       <c r="L1528" t="n">
         <v>4.91</v>
@@ -67704,7 +67704,7 @@
         <v>8.289999999999999</v>
       </c>
       <c r="K1529" t="n">
-        <v>307562</v>
+        <v>307559</v>
       </c>
       <c r="L1529" t="n">
         <v>4.91</v>
@@ -67924,7 +67924,7 @@
         <v>8.32</v>
       </c>
       <c r="K1534" t="n">
-        <v>210003</v>
+        <v>209988</v>
       </c>
       <c r="L1534" t="n">
         <v>4.91</v>
@@ -67968,7 +67968,7 @@
         <v>8.31</v>
       </c>
       <c r="K1535" t="n">
-        <v>11721801</v>
+        <v>41090</v>
       </c>
       <c r="L1535" t="n">
         <v>4.91</v>
@@ -68220,7 +68220,7 @@
         </is>
       </c>
       <c r="G1541" t="n">
-        <v>8.609999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="H1541" t="n">
         <v>8.619999999999999</v>
@@ -68232,7 +68232,7 @@
         <v>8.609999999999999</v>
       </c>
       <c r="K1541" t="n">
-        <v>34777</v>
+        <v>33728</v>
       </c>
       <c r="L1541" t="n">
         <v>4.91</v>
@@ -69012,7 +69012,7 @@
         </is>
       </c>
       <c r="G1559" t="n">
-        <v>7.94</v>
+        <v>7.95</v>
       </c>
       <c r="H1559" t="n">
         <v>8.08</v>
@@ -69596,7 +69596,7 @@
         <v>8.1</v>
       </c>
       <c r="K1572" t="n">
-        <v>13113558</v>
+        <v>10574</v>
       </c>
       <c r="L1572" t="n">
         <v>4.91</v>
@@ -74248,13 +74248,13 @@
         </is>
       </c>
       <c r="G1678" t="n">
-        <v>6.85</v>
+        <v>6.93</v>
       </c>
       <c r="H1678" t="n">
-        <v>6.85</v>
+        <v>6.93</v>
       </c>
       <c r="I1678" t="n">
-        <v>6.85</v>
+        <v>6.74</v>
       </c>
       <c r="J1678" t="n">
         <v>6.85</v>
@@ -84028,7 +84028,7 @@
         <v>14.17</v>
       </c>
       <c r="K1900" t="n">
-        <v>5104</v>
+        <v>5154</v>
       </c>
       <c r="L1900" t="n">
         <v>14.5</v>
@@ -84072,7 +84072,7 @@
         <v>14.45</v>
       </c>
       <c r="K1901" t="n">
-        <v>3899</v>
+        <v>3849</v>
       </c>
       <c r="L1901" t="n">
         <v>14.5</v>
@@ -86096,7 +86096,7 @@
         <v>14.04</v>
       </c>
       <c r="K1947" t="n">
-        <v>167</v>
+        <v>215</v>
       </c>
       <c r="L1947" t="n">
         <v>14.5</v>
@@ -86140,7 +86140,7 @@
         <v>14</v>
       </c>
       <c r="K1948" t="n">
-        <v>691</v>
+        <v>643</v>
       </c>
       <c r="L1948" t="n">
         <v>14.5</v>
@@ -87504,7 +87504,7 @@
         <v>14.06</v>
       </c>
       <c r="K1979" t="n">
-        <v>1289</v>
+        <v>819</v>
       </c>
       <c r="L1979" t="n">
         <v>14.5</v>
@@ -88296,7 +88296,7 @@
         <v>14.04</v>
       </c>
       <c r="K1997" t="n">
-        <v>1763</v>
+        <v>1457</v>
       </c>
       <c r="L1997" t="n">
         <v>14.5</v>
@@ -91112,7 +91112,7 @@
         <v>14.11</v>
       </c>
       <c r="K2061" t="n">
-        <v>953</v>
+        <v>969</v>
       </c>
       <c r="L2061" t="n">
         <v>14.5</v>
@@ -91156,7 +91156,7 @@
         <v>14.05</v>
       </c>
       <c r="K2062" t="n">
-        <v>629</v>
+        <v>613</v>
       </c>
       <c r="L2062" t="n">
         <v>14.5</v>
@@ -91860,7 +91860,7 @@
         <v>13.98</v>
       </c>
       <c r="K2078" t="n">
-        <v>7907</v>
+        <v>7985</v>
       </c>
       <c r="L2078" t="n">
         <v>14.5</v>
@@ -91904,7 +91904,7 @@
         <v>13.91</v>
       </c>
       <c r="K2079" t="n">
-        <v>6117</v>
+        <v>6039</v>
       </c>
       <c r="L2079" t="n">
         <v>14.5</v>
@@ -92168,7 +92168,7 @@
         <v>14.17</v>
       </c>
       <c r="K2085" t="n">
-        <v>1266</v>
+        <v>1364</v>
       </c>
       <c r="L2085" t="n">
         <v>14.5</v>
@@ -92212,7 +92212,7 @@
         <v>14.23</v>
       </c>
       <c r="K2086" t="n">
-        <v>14544</v>
+        <v>14446</v>
       </c>
       <c r="L2086" t="n">
         <v>14.5</v>

</xml_diff>